<commit_message>
Update dashboard and version control tracker
</commit_message>
<xml_diff>
--- a/SOP-Version-Control-Log.xlsx
+++ b/SOP-Version-Control-Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\adeola\clinical-data-portfolio\sop-qsm-version-control-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3331ECCA-2031-465D-98F3-2BDAA146CFFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817D0E79-04C7-4EE3-A528-BDA7F4790E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{4E23EB7A-6D0F-4A01-ACFF-5EA9D42706E6}"/>
   </bookViews>
@@ -498,13 +498,13 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>92</c:v>
+                  <c:v>91</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>105</c:v>
+                  <c:v>104</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>160</c:v>
+                  <c:v>159</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -552,14 +552,14 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-GB"/>
+                  <a:rPr lang="en-GB" b="1"/>
                   <a:t>SOP</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:rPr lang="en-GB" b="1" baseline="0"/>
                   <a:t> Number</a:t>
                 </a:r>
-                <a:endParaRPr lang="en-GB"/>
+                <a:endParaRPr lang="en-GB" b="1"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -593,7 +593,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -679,7 +679,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-GB">
+                  <a:rPr lang="en-GB" b="1">
                     <a:ln>
                       <a:noFill/>
                     </a:ln>
@@ -687,14 +687,14 @@
                   <a:t>Days</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-GB" baseline="0">
+                  <a:rPr lang="en-GB" b="1" baseline="0">
                     <a:ln>
                       <a:noFill/>
                     </a:ln>
                   </a:rPr>
                   <a:t> Until Review</a:t>
                 </a:r>
-                <a:endParaRPr lang="en-GB">
+                <a:endParaRPr lang="en-GB" b="1">
                   <a:ln>
                     <a:noFill/>
                   </a:ln>
@@ -735,7 +735,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="F2" s="28">
         <f ca="1">E2-TODAY()</f>
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="F3" s="28">
         <f t="shared" ref="F3:F4" ca="1" si="0">E3-TODAY()</f>
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="F4" s="28">
         <f t="shared" ca="1" si="0"/>
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>